<commit_message>
feat: complete attendance, leave, payroll and announcement modules
</commit_message>
<xml_diff>
--- a/Depo EMP List.xlsx
+++ b/Depo EMP List.xlsx
@@ -1,31 +1,62 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/792DF01DACF152E5/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/792df01dacf152e5/Desktop/BINDU-EMS/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{226505EE-3F1F-43A6-B287-61D8CEEEDA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="8_{226505EE-3F1F-43A6-B287-61D8CEEEDA6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC7A274F-EB23-403F-94E1-3F3FCD85937A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" calcCompleted="0"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xda="http://schemas.microsoft.com/office/spreadsheetml/2017/dynamicarray">
+  <metadataTypes count="1">
+    <metadataType name="XLDAPR" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1" cellMeta="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLDAPR" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{bdbb8cdc-fa1e-496e-a857-3c3f30c029c3}">
+          <xda:dynamicArrayProperties fDynamic="1" fCollapsed="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <cellMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </cellMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="380" uniqueCount="218">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="382" uniqueCount="220">
   <si>
     <t>ID NO</t>
   </si>
@@ -679,6 +710,12 @@
   </si>
   <si>
     <t>SALEM</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                            Latitude / Longitude</t>
+  </si>
+  <si>
+    <t>11.199608334152948, 75.83228955147506</t>
   </si>
 </sst>
 </file>
@@ -805,7 +842,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -819,6 +856,10 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1101,7 +1142,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:E77"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.88671875" customWidth="1"/>
@@ -1109,9 +1150,15 @@
     <col min="3" max="3" width="19.5546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="15.44140625" customWidth="1"/>
     <col min="5" max="5" width="18.33203125" customWidth="1"/>
+    <col min="7" max="7" width="44" customWidth="1"/>
+    <col min="8" max="8" width="30.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H1" s="11"/>
+      <c r="I1" s="11"/>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1127,8 +1174,13 @@
       <c r="E2" s="1" t="s">
         <v>130</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G2" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="H2" s="12"/>
+      <c r="I2" s="11"/>
+    </row>
+    <row r="3" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>162</v>
       </c>
@@ -1144,8 +1196,14 @@
       <c r="E3" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G3" s="10"/>
+      <c r="H3" s="11" cm="1">
+        <f t="array" aca="1" ref="H3" ca="1">H3:H67</f>
+        <v>0</v>
+      </c>
+      <c r="I3" s="11"/>
+    </row>
+    <row r="4" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
         <v>118</v>
       </c>
@@ -1161,8 +1219,11 @@
       <c r="E4" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G4" s="10"/>
+      <c r="H4" s="11"/>
+      <c r="I4" s="11"/>
+    </row>
+    <row r="5" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>169</v>
       </c>
@@ -1178,8 +1239,11 @@
       <c r="E5" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G5" s="10"/>
+      <c r="H5" s="11"/>
+      <c r="I5" s="11"/>
+    </row>
+    <row r="6" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>170</v>
       </c>
@@ -1195,8 +1259,11 @@
       <c r="E6" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G6" s="10"/>
+      <c r="H6" s="11"/>
+      <c r="I6" s="11"/>
+    </row>
+    <row r="7" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
         <v>171</v>
       </c>
@@ -1212,8 +1279,11 @@
       <c r="E7" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G7" s="10"/>
+      <c r="H7" s="11"/>
+      <c r="I7" s="11"/>
+    </row>
+    <row r="8" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
         <v>123</v>
       </c>
@@ -1229,8 +1299,11 @@
       <c r="E8" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G8" s="10"/>
+      <c r="H8" s="11"/>
+      <c r="I8" s="11"/>
+    </row>
+    <row r="9" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="2" t="s">
         <v>172</v>
       </c>
@@ -1246,8 +1319,11 @@
       <c r="E9" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G9" s="10"/>
+      <c r="H9" s="11"/>
+      <c r="I9" s="11"/>
+    </row>
+    <row r="10" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="2" t="s">
         <v>154</v>
       </c>
@@ -1263,8 +1339,11 @@
       <c r="E10" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G10" s="10"/>
+      <c r="H10" s="11"/>
+      <c r="I10" s="11"/>
+    </row>
+    <row r="11" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="2" t="s">
         <v>124</v>
       </c>
@@ -1280,8 +1359,11 @@
       <c r="E11" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G11" s="10"/>
+      <c r="H11" s="11"/>
+      <c r="I11" s="11"/>
+    </row>
+    <row r="12" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="2" t="s">
         <v>173</v>
       </c>
@@ -1297,8 +1379,11 @@
       <c r="E12" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G12" s="10"/>
+      <c r="H12" s="11"/>
+      <c r="I12" s="11"/>
+    </row>
+    <row r="13" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>168</v>
       </c>
@@ -1314,8 +1399,11 @@
       <c r="E13" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G13" s="10"/>
+      <c r="H13" s="11"/>
+      <c r="I13" s="11"/>
+    </row>
+    <row r="14" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="2" t="s">
         <v>117</v>
       </c>
@@ -1331,8 +1419,11 @@
       <c r="E14" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G14" s="10"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+    </row>
+    <row r="15" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="2" t="s">
         <v>115</v>
       </c>
@@ -1348,8 +1439,11 @@
       <c r="E15" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G15" s="10"/>
+      <c r="H15" s="11"/>
+      <c r="I15" s="11"/>
+    </row>
+    <row r="16" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A16" s="2" t="s">
         <v>174</v>
       </c>
@@ -1365,8 +1459,11 @@
       <c r="E16" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G16" s="10"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A17" s="2" t="s">
         <v>175</v>
       </c>
@@ -1382,8 +1479,11 @@
       <c r="E17" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G17" s="10"/>
+      <c r="H17" s="11"/>
+      <c r="I17" s="11"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A18" s="2" t="s">
         <v>164</v>
       </c>
@@ -1399,8 +1499,11 @@
       <c r="E18" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G18" s="10"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A19" s="2" t="s">
         <v>155</v>
       </c>
@@ -1416,8 +1519,11 @@
       <c r="E19" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G19" s="10"/>
+      <c r="H19" s="11"/>
+      <c r="I19" s="11"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
         <v>156</v>
       </c>
@@ -1433,8 +1539,11 @@
       <c r="E20" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G20" s="10"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A21" s="2" t="s">
         <v>176</v>
       </c>
@@ -1450,8 +1559,11 @@
       <c r="E21" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G21" s="10"/>
+      <c r="H21" s="11"/>
+      <c r="I21" s="11"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A22" s="2" t="s">
         <v>177</v>
       </c>
@@ -1467,8 +1579,11 @@
       <c r="E22" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G22" s="10"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A23" s="2" t="s">
         <v>178</v>
       </c>
@@ -1484,8 +1599,11 @@
       <c r="E23" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G23" s="10"/>
+      <c r="H23" s="11"/>
+      <c r="I23" s="11"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A24" s="2" t="s">
         <v>114</v>
       </c>
@@ -1501,8 +1619,11 @@
       <c r="E24" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G24" s="10"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A25" s="2" t="s">
         <v>165</v>
       </c>
@@ -1518,8 +1639,11 @@
       <c r="E25" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G25" s="10"/>
+      <c r="H25" s="11"/>
+      <c r="I25" s="11"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A26" s="2" t="s">
         <v>179</v>
       </c>
@@ -1535,8 +1659,11 @@
       <c r="E26" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G26" s="10"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A27" s="2" t="s">
         <v>158</v>
       </c>
@@ -1552,8 +1679,11 @@
       <c r="E27" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G27" s="10"/>
+      <c r="H27" s="11"/>
+      <c r="I27" s="11"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A28" s="2" t="s">
         <v>180</v>
       </c>
@@ -1569,8 +1699,11 @@
       <c r="E28" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G28" s="10"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A29" s="2" t="s">
         <v>181</v>
       </c>
@@ -1586,8 +1719,11 @@
       <c r="E29" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G29" s="10"/>
+      <c r="H29" s="11"/>
+      <c r="I29" s="11"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
         <v>163</v>
       </c>
@@ -1603,8 +1739,11 @@
       <c r="E30" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G30" s="10"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A31" s="2" t="s">
         <v>182</v>
       </c>
@@ -1620,8 +1759,11 @@
       <c r="E31" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G31" s="10"/>
+      <c r="H31" s="11"/>
+      <c r="I31" s="11"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
         <v>160</v>
       </c>
@@ -1637,8 +1779,11 @@
       <c r="E32" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G32" s="10"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+    </row>
+    <row r="33" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A33" s="2" t="s">
         <v>194</v>
       </c>
@@ -1654,8 +1799,11 @@
       <c r="E33" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G33" s="10"/>
+      <c r="H33" s="11"/>
+      <c r="I33" s="11"/>
+    </row>
+    <row r="34" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A34" s="2" t="s">
         <v>120</v>
       </c>
@@ -1671,8 +1819,11 @@
       <c r="E34" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G34" s="10"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+    </row>
+    <row r="35" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A35" s="2" t="s">
         <v>183</v>
       </c>
@@ -1688,8 +1839,11 @@
       <c r="E35" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G35" s="10"/>
+      <c r="H35" s="11"/>
+      <c r="I35" s="11"/>
+    </row>
+    <row r="36" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A36" s="2" t="s">
         <v>184</v>
       </c>
@@ -1705,8 +1859,11 @@
       <c r="E36" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G36" s="10"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+    </row>
+    <row r="37" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A37" s="2" t="s">
         <v>125</v>
       </c>
@@ -1722,8 +1879,11 @@
       <c r="E37" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G37" s="10"/>
+      <c r="H37" s="11"/>
+      <c r="I37" s="11"/>
+    </row>
+    <row r="38" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A38" s="2" t="s">
         <v>185</v>
       </c>
@@ -1739,8 +1899,11 @@
       <c r="E38" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G38" s="10"/>
+      <c r="H38" s="11"/>
+      <c r="I38" s="11"/>
+    </row>
+    <row r="39" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A39" s="2" t="s">
         <v>121</v>
       </c>
@@ -1756,8 +1919,11 @@
       <c r="E39" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G39" s="10"/>
+      <c r="H39" s="11"/>
+      <c r="I39" s="11"/>
+    </row>
+    <row r="40" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="2" t="s">
         <v>186</v>
       </c>
@@ -1773,8 +1939,11 @@
       <c r="E40" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G40" s="10"/>
+      <c r="H40" s="11"/>
+      <c r="I40" s="11"/>
+    </row>
+    <row r="41" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A41" s="2" t="s">
         <v>119</v>
       </c>
@@ -1790,8 +1959,11 @@
       <c r="E41" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G41" s="10"/>
+      <c r="H41" s="11"/>
+      <c r="I41" s="11"/>
+    </row>
+    <row r="42" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A42" s="2" t="s">
         <v>187</v>
       </c>
@@ -1807,8 +1979,11 @@
       <c r="E42" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G42" s="10"/>
+      <c r="H42" s="11"/>
+      <c r="I42" s="11"/>
+    </row>
+    <row r="43" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A43" s="2" t="s">
         <v>127</v>
       </c>
@@ -1824,8 +1999,11 @@
       <c r="E43" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G43" s="10"/>
+      <c r="H43" s="11"/>
+      <c r="I43" s="11"/>
+    </row>
+    <row r="44" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A44" s="2" t="s">
         <v>188</v>
       </c>
@@ -1841,8 +2019,11 @@
       <c r="E44" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G44" s="10"/>
+      <c r="H44" s="11"/>
+      <c r="I44" s="11"/>
+    </row>
+    <row r="45" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A45" s="2" t="s">
         <v>122</v>
       </c>
@@ -1858,8 +2039,11 @@
       <c r="E45" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G45" s="10"/>
+      <c r="H45" s="11"/>
+      <c r="I45" s="11"/>
+    </row>
+    <row r="46" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A46" s="2" t="s">
         <v>189</v>
       </c>
@@ -1875,8 +2059,11 @@
       <c r="E46" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G46" s="10"/>
+      <c r="H46" s="11"/>
+      <c r="I46" s="11"/>
+    </row>
+    <row r="47" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A47" s="2" t="s">
         <v>126</v>
       </c>
@@ -1892,8 +2079,11 @@
       <c r="E47" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G47" s="10"/>
+      <c r="H47" s="11"/>
+      <c r="I47" s="11"/>
+    </row>
+    <row r="48" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A48" s="2" t="s">
         <v>190</v>
       </c>
@@ -1909,8 +2099,11 @@
       <c r="E48" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G48" s="10"/>
+      <c r="H48" s="11"/>
+      <c r="I48" s="11"/>
+    </row>
+    <row r="49" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A49" s="2" t="s">
         <v>191</v>
       </c>
@@ -1926,8 +2119,11 @@
       <c r="E49" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G49" s="10"/>
+      <c r="H49" s="11"/>
+      <c r="I49" s="11"/>
+    </row>
+    <row r="50" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A50" s="2" t="s">
         <v>192</v>
       </c>
@@ -1943,8 +2139,11 @@
       <c r="E50" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G50" s="10"/>
+      <c r="H50" s="11"/>
+      <c r="I50" s="11"/>
+    </row>
+    <row r="51" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A51" s="2" t="s">
         <v>193</v>
       </c>
@@ -1960,8 +2159,11 @@
       <c r="E51" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G51" s="10"/>
+      <c r="H51" s="11"/>
+      <c r="I51" s="11"/>
+    </row>
+    <row r="52" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A52" s="2" t="s">
         <v>157</v>
       </c>
@@ -1977,8 +2179,11 @@
       <c r="E52" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G52" s="10"/>
+      <c r="H52" s="11"/>
+      <c r="I52" s="11"/>
+    </row>
+    <row r="53" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A53" s="2" t="s">
         <v>195</v>
       </c>
@@ -1994,8 +2199,11 @@
       <c r="E53" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G53" s="10"/>
+      <c r="H53" s="11"/>
+      <c r="I53" s="11"/>
+    </row>
+    <row r="54" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A54" s="2" t="s">
         <v>167</v>
       </c>
@@ -2011,8 +2219,11 @@
       <c r="E54" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G54" s="10"/>
+      <c r="H54" s="11"/>
+      <c r="I54" s="11"/>
+    </row>
+    <row r="55" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A55" s="2" t="s">
         <v>196</v>
       </c>
@@ -2028,8 +2239,11 @@
       <c r="E55" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G55" s="10"/>
+      <c r="H55" s="11"/>
+      <c r="I55" s="11"/>
+    </row>
+    <row r="56" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A56" s="2" t="s">
         <v>197</v>
       </c>
@@ -2045,8 +2259,11 @@
       <c r="E56" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G56" s="10"/>
+      <c r="H56" s="11"/>
+      <c r="I56" s="11"/>
+    </row>
+    <row r="57" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A57" s="2" t="s">
         <v>198</v>
       </c>
@@ -2062,8 +2279,11 @@
       <c r="E57" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G57" s="10"/>
+      <c r="H57" s="11"/>
+      <c r="I57" s="11"/>
+    </row>
+    <row r="58" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
         <v>199</v>
       </c>
@@ -2079,8 +2299,11 @@
       <c r="E58" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G58" s="10"/>
+      <c r="H58" s="11"/>
+      <c r="I58" s="11"/>
+    </row>
+    <row r="59" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
         <v>200</v>
       </c>
@@ -2096,8 +2319,11 @@
       <c r="E59" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G59" s="10"/>
+      <c r="H59" s="11"/>
+      <c r="I59" s="11"/>
+    </row>
+    <row r="60" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
         <v>166</v>
       </c>
@@ -2113,8 +2339,13 @@
       <c r="E60" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G60" s="10" t="s">
+        <v>219</v>
+      </c>
+      <c r="H60" s="11"/>
+      <c r="I60" s="11"/>
+    </row>
+    <row r="61" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A61" s="2" t="s">
         <v>201</v>
       </c>
@@ -2130,8 +2361,11 @@
       <c r="E61" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G61" s="10"/>
+      <c r="H61" s="11"/>
+      <c r="I61" s="11"/>
+    </row>
+    <row r="62" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A62" s="2" t="s">
         <v>159</v>
       </c>
@@ -2147,8 +2381,11 @@
       <c r="E62" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G62" s="10"/>
+      <c r="H62" s="11"/>
+      <c r="I62" s="11"/>
+    </row>
+    <row r="63" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A63" s="2" t="s">
         <v>202</v>
       </c>
@@ -2164,8 +2401,11 @@
       <c r="E63" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G63" s="10"/>
+      <c r="H63" s="11"/>
+      <c r="I63" s="11"/>
+    </row>
+    <row r="64" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A64" s="2" t="s">
         <v>203</v>
       </c>
@@ -2181,8 +2421,11 @@
       <c r="E64" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G64" s="10"/>
+      <c r="H64" s="11"/>
+      <c r="I64" s="11"/>
+    </row>
+    <row r="65" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
         <v>204</v>
       </c>
@@ -2198,8 +2441,11 @@
       <c r="E65" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G65" s="10"/>
+      <c r="H65" s="11"/>
+      <c r="I65" s="11"/>
+    </row>
+    <row r="66" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A66" s="2" t="s">
         <v>205</v>
       </c>
@@ -2215,8 +2461,11 @@
       <c r="E66" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G66" s="10"/>
+      <c r="H66" s="11"/>
+      <c r="I66" s="11"/>
+    </row>
+    <row r="67" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A67" s="2" t="s">
         <v>206</v>
       </c>
@@ -2232,8 +2481,11 @@
       <c r="E67" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G67" s="10"/>
+      <c r="H67" s="11"/>
+      <c r="I67" s="11"/>
+    </row>
+    <row r="68" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A68" s="2" t="s">
         <v>207</v>
       </c>
@@ -2249,8 +2501,11 @@
       <c r="E68" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G68" s="10"/>
+      <c r="H68" s="11"/>
+      <c r="I68" s="11"/>
+    </row>
+    <row r="69" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A69" s="2" t="s">
         <v>208</v>
       </c>
@@ -2266,8 +2521,11 @@
       <c r="E69" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G69" s="10"/>
+      <c r="H69" s="11"/>
+      <c r="I69" s="11"/>
+    </row>
+    <row r="70" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A70" s="2" t="s">
         <v>209</v>
       </c>
@@ -2283,8 +2541,11 @@
       <c r="E70" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G70" s="10"/>
+      <c r="H70" s="11"/>
+      <c r="I70" s="11"/>
+    </row>
+    <row r="71" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
         <v>210</v>
       </c>
@@ -2300,8 +2561,11 @@
       <c r="E71" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G71" s="10"/>
+      <c r="H71" s="11"/>
+      <c r="I71" s="11"/>
+    </row>
+    <row r="72" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A72" s="2" t="s">
         <v>211</v>
       </c>
@@ -2317,8 +2581,11 @@
       <c r="E72" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G72" s="10"/>
+      <c r="H72" s="11"/>
+      <c r="I72" s="11"/>
+    </row>
+    <row r="73" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A73" s="2" t="s">
         <v>212</v>
       </c>
@@ -2334,8 +2601,11 @@
       <c r="E73" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G73" s="10"/>
+      <c r="H73" s="11"/>
+      <c r="I73" s="11"/>
+    </row>
+    <row r="74" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A74" s="2" t="s">
         <v>213</v>
       </c>
@@ -2351,8 +2621,11 @@
       <c r="E74" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G74" s="10"/>
+      <c r="H74" s="11"/>
+      <c r="I74" s="11"/>
+    </row>
+    <row r="75" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A75" s="2" t="s">
         <v>116</v>
       </c>
@@ -2368,8 +2641,11 @@
       <c r="E75" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G75" s="10"/>
+      <c r="H75" s="11"/>
+      <c r="I75" s="11"/>
+    </row>
+    <row r="76" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A76" s="2" t="s">
         <v>214</v>
       </c>
@@ -2385,8 +2661,11 @@
       <c r="E76" s="5" t="s">
         <v>128</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="G76" s="10"/>
+      <c r="H76" s="11"/>
+      <c r="I76" s="11"/>
+    </row>
+    <row r="77" spans="1:9" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A77" s="2" t="s">
         <v>215</v>
       </c>
@@ -2402,6 +2681,13 @@
       <c r="E77" s="5" t="s">
         <v>128</v>
       </c>
+      <c r="G77" s="10"/>
+      <c r="H77" s="11"/>
+      <c r="I77" s="11"/>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="H78" s="11"/>
+      <c r="I78" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>